<commit_message>
Update rho 0.1 lower-bound comparison results
</commit_message>
<xml_diff>
--- a/results/by_density/rho_0.1/msig_vs_lower_bound_rho_0.1.xlsx
+++ b/results/by_density/rho_0.1/msig_vs_lower_bound_rho_0.1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra9c98e454be64241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Row" sheetId="2" r:id="Rf62a39352a0049f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instance_Comparison" sheetId="3" r:id="R8a5807cb69364762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7bfb7069bef6474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Row" sheetId="2" r:id="Rbc8ca3073fee4654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instance_Comparison" sheetId="3" r:id="R503bd9d29551447c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -478,7 +478,7 @@
       </x:c>
       <x:c r="B4" s="44" t="n">
         <x:f>AVERAGEIF(Instance_Comparison!B2:B577,A4,Instance_Comparison!E2:E577)</x:f>
-        <x:v>6.446988160726457</x:v>
+        <x:v>6.389117790356086</x:v>
       </x:c>
       <x:c r="C4" s="45" t="n">
         <x:f>COUNTIFS(Instance_Comparison!B2:B577,A4,Instance_Comparison!F2:F577,"YES")</x:f>
@@ -495,7 +495,7 @@
       </x:c>
       <x:c r="B5" s="44" t="n">
         <x:f>AVERAGEIF(Instance_Comparison!B2:B577,A5,Instance_Comparison!E2:E577)</x:f>
-        <x:v>6.053336346624803</x:v>
+        <x:v>5.98506186292515</x:v>
       </x:c>
       <x:c r="C5" s="45" t="n">
         <x:f>COUNTIFS(Instance_Comparison!B2:B577,A5,Instance_Comparison!F2:F577,"YES")</x:f>
@@ -512,7 +512,7 @@
       </x:c>
       <x:c r="B6" s="48" t="n">
         <x:f>AVERAGE(Instance_Comparison!E2:E577)</x:f>
-        <x:v>5.47249119309464</x:v>
+        <x:v>5.440954979577135</x:v>
       </x:c>
       <x:c r="C6" s="49" t="n">
         <x:f>COUNTIF(Instance_Comparison!F2:F577,"YES")</x:f>
@@ -573,15 +573,15 @@
       </x:c>
       <x:c r="D2" s="49" t="str">
         <x:f>TEXT(Summary!B4,"0.00")&amp;"% ("&amp;Summary!C4&amp;"/"&amp;Summary!D4&amp;")"</x:f>
-        <x:v>6.45% (13/144)</x:v>
+        <x:v>6.39% (13/144)</x:v>
       </x:c>
       <x:c r="E2" s="49" t="str">
         <x:f>TEXT(Summary!B5,"0.00")&amp;"% ("&amp;Summary!C5&amp;"/"&amp;Summary!D5&amp;")"</x:f>
-        <x:v>6.05% (9/144)</x:v>
+        <x:v>5.99% (9/144)</x:v>
       </x:c>
       <x:c r="F2" s="50" t="str">
         <x:f>TEXT(Summary!B6,"0.00")&amp;"% ("&amp;Summary!C6&amp;"/"&amp;Summary!D6&amp;")"</x:f>
-        <x:v>5.47% (153/576)</x:v>
+        <x:v>5.44% (153/576)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -752,11 +752,11 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D6" s="28" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E6" s="39" t="n">
         <x:f>(C6-D6)/C6*100</x:f>
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F6" s="28" t="str">
         <x:f>IF(C6=D6,"YES","NO")</x:f>
@@ -2600,11 +2600,11 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="D72" s="28" t="n">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E72" s="39" t="n">
         <x:f>(C72-D72)/C72*100</x:f>
-        <x:v>9.67741935483871</x:v>
+        <x:v>6.451612903225806</x:v>
       </x:c>
       <x:c r="F72" s="28" t="str">
         <x:f>IF(C72=D72,"YES","NO")</x:f>
@@ -3188,11 +3188,11 @@
         <x:v>849</x:v>
       </x:c>
       <x:c r="D93" s="28" t="n">
-        <x:v>814</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="E93" s="39" t="n">
         <x:f>(C93-D93)/C93*100</x:f>
-        <x:v>4.122497055359246</x:v>
+        <x:v>4.004711425206125</x:v>
       </x:c>
       <x:c r="F93" s="28" t="str">
         <x:f>IF(C93=D93,"YES","NO")</x:f>
@@ -7248,11 +7248,11 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D238" s="28" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E238" s="39" t="n">
         <x:f>(C238-D238)/C238*100</x:f>
-        <x:v>10</x:v>
+        <x:v>6.666666666666667</x:v>
       </x:c>
       <x:c r="F238" s="28" t="str">
         <x:f>IF(C238=D238,"YES","NO")</x:f>
@@ -8200,11 +8200,11 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="D272" s="28" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E272" s="39" t="n">
         <x:f>(C272-D272)/C272*100</x:f>
-        <x:v>12.5</x:v>
+        <x:v>6.25</x:v>
       </x:c>
       <x:c r="F272" s="28" t="str">
         <x:f>IF(C272=D272,"YES","NO")</x:f>
@@ -8564,11 +8564,11 @@
         <x:v>860</x:v>
       </x:c>
       <x:c r="D285" s="28" t="n">
-        <x:v>803</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="E285" s="39" t="n">
         <x:f>(C285-D285)/C285*100</x:f>
-        <x:v>6.627906976744185</x:v>
+        <x:v>6.511627906976744</x:v>
       </x:c>
       <x:c r="F285" s="28" t="str">
         <x:f>IF(C285=D285,"YES","NO")</x:f>
@@ -14052,11 +14052,11 @@
         <x:v>822</x:v>
       </x:c>
       <x:c r="D481" s="28" t="n">
-        <x:v>768</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="E481" s="39" t="n">
         <x:f>(C481-D481)/C481*100</x:f>
-        <x:v>6.569343065693431</x:v>
+        <x:v>6.447688564476886</x:v>
       </x:c>
       <x:c r="F481" s="28" t="str">
         <x:f>IF(C481=D481,"YES","NO")</x:f>

</xml_diff>